<commit_message>
feat: ordena colunas e publica paginas e relatorios estaticos
</commit_message>
<xml_diff>
--- a/DADOS.xlsx
+++ b/DADOS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://justicagovbr-my.sharepoint.com/personal/marcelo_cortez_mj_gov_br1/Documents/1. SENAPPEN/2. OUVIDORIA/GITHUB/PARAMETROS MINIMOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="500" documentId="11_C2318B871671820C540791CC0C0EFCB85A7F69AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4BB34C04-656A-4D0C-95AE-47E7C66E1053}"/>
+  <xr:revisionPtr revIDLastSave="520" documentId="11_C2318B871671820C540791CC0C0EFCB85A7F69AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C5ABA7F-6B2D-4B87-9667-78C2E164606E}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1771,11 +1771,25 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="125">
+  <dxfs count="87">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFE2F0D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFF4CCCC"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1818,292 +1832,6 @@
       <fill>
         <patternFill patternType="solid">
           <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF375623"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFFF2CC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFF4CCCC"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFE2F0D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4137,7 +3865,7 @@
         <v>150</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>99</v>
@@ -4147,15 +3875,15 @@
       </c>
       <c r="F31" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G31" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H31" s="3" t="str">
         <f t="shared" si="2"/>
-        <v>Não instituída</v>
+        <v>Instituída</v>
       </c>
       <c r="I31" s="3" t="s">
         <v>521</v>
@@ -6468,7 +6196,7 @@
         <v>150</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>182</v>
@@ -6478,10 +6206,10 @@
       </c>
       <c r="F31" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>183</v>
@@ -6491,7 +6219,7 @@
       </c>
       <c r="J31" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K31" s="3" t="s">
         <v>522</v>
@@ -6534,7 +6262,7 @@
       </c>
       <c r="W31" s="3">
         <f t="shared" si="5"/>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="X31" s="3" t="s">
         <v>96</v>
@@ -6785,57 +6513,57 @@
     <mergeCell ref="W4:X4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C34">
-    <cfRule type="expression" dxfId="124" priority="1">
+    <cfRule type="expression" dxfId="86" priority="1">
       <formula>C7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="123" priority="2">
+    <cfRule type="expression" dxfId="85" priority="2">
       <formula>C7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="122" priority="3">
+    <cfRule type="expression" dxfId="84" priority="3">
       <formula>OR(C7="Não atende",C7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:G34">
-    <cfRule type="expression" dxfId="121" priority="4">
+    <cfRule type="expression" dxfId="83" priority="4">
       <formula>G7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="120" priority="5">
+    <cfRule type="expression" dxfId="82" priority="5">
       <formula>G7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="119" priority="6">
+    <cfRule type="expression" dxfId="81" priority="6">
       <formula>OR(G7="Não atende",G7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7:K34">
-    <cfRule type="expression" dxfId="118" priority="7">
+    <cfRule type="expression" dxfId="80" priority="7">
       <formula>K7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="117" priority="8">
+    <cfRule type="expression" dxfId="79" priority="8">
       <formula>K7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="116" priority="9">
+    <cfRule type="expression" dxfId="78" priority="9">
       <formula>OR(K7="Não atende",K7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O7:O34">
-    <cfRule type="expression" dxfId="115" priority="10">
+    <cfRule type="expression" dxfId="77" priority="10">
       <formula>O7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="114" priority="11">
+    <cfRule type="expression" dxfId="76" priority="11">
       <formula>O7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="113" priority="12">
+    <cfRule type="expression" dxfId="75" priority="12">
       <formula>OR(O7="Não atende",O7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S7:S34">
-    <cfRule type="expression" dxfId="112" priority="13">
+    <cfRule type="expression" dxfId="74" priority="13">
       <formula>S7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="111" priority="14">
+    <cfRule type="expression" dxfId="73" priority="14">
       <formula>S7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="110" priority="15">
+    <cfRule type="expression" dxfId="72" priority="15">
       <formula>OR(S7="Não atende",S7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7987,7 +7715,7 @@
         <v>150</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>235</v>
@@ -7997,10 +7725,10 @@
       </c>
       <c r="F31" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>232</v>
@@ -8010,11 +7738,11 @@
       </c>
       <c r="J31" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="K31" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>96</v>
@@ -8154,24 +7882,24 @@
     <mergeCell ref="K4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C34">
-    <cfRule type="expression" dxfId="109" priority="1">
+    <cfRule type="expression" dxfId="71" priority="1">
       <formula>C7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="108" priority="2">
+    <cfRule type="expression" dxfId="70" priority="2">
       <formula>C7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="107" priority="3">
+    <cfRule type="expression" dxfId="69" priority="3">
       <formula>OR(C7="Não atende",C7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:G34">
-    <cfRule type="expression" dxfId="106" priority="4">
+    <cfRule type="expression" dxfId="68" priority="4">
       <formula>G7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="105" priority="5">
+    <cfRule type="expression" dxfId="67" priority="5">
       <formula>G7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="104" priority="6">
+    <cfRule type="expression" dxfId="66" priority="6">
       <formula>OR(G7="Não atende",G7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10733,7 +10461,7 @@
         <v>150</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>73</v>
@@ -10743,10 +10471,10 @@
       </c>
       <c r="F31" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>73</v>
@@ -10756,10 +10484,10 @@
       </c>
       <c r="J31" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K31" s="3" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="L31" s="5" t="s">
         <v>73</v>
@@ -10769,10 +10497,10 @@
       </c>
       <c r="N31" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O31" s="3" t="s">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="P31" s="5" t="s">
         <v>278</v>
@@ -10782,10 +10510,10 @@
       </c>
       <c r="R31" s="3">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="T31" s="5" t="s">
         <v>274</v>
@@ -10795,10 +10523,10 @@
       </c>
       <c r="V31" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="W31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="X31" s="5" t="s">
         <v>297</v>
@@ -10808,11 +10536,11 @@
       </c>
       <c r="Z31" s="3">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AA31" s="3">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="AB31" s="3" t="s">
         <v>96</v>
@@ -11109,68 +10837,68 @@
     <mergeCell ref="AA4:AB4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C34">
-    <cfRule type="expression" dxfId="103" priority="1">
+    <cfRule type="expression" dxfId="65" priority="1">
       <formula>C7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="102" priority="2">
+    <cfRule type="expression" dxfId="64" priority="2">
       <formula>C7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="101" priority="3">
+    <cfRule type="expression" dxfId="63" priority="3">
       <formula>OR(C7="Não atende",C7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:G34">
-    <cfRule type="expression" dxfId="100" priority="4">
+    <cfRule type="expression" dxfId="62" priority="4">
       <formula>G7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="99" priority="5">
+    <cfRule type="expression" dxfId="61" priority="5">
       <formula>G7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="98" priority="6">
+    <cfRule type="expression" dxfId="60" priority="6">
       <formula>OR(G7="Não atende",G7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7:K34">
-    <cfRule type="expression" dxfId="97" priority="7">
+    <cfRule type="expression" dxfId="59" priority="7">
       <formula>K7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="96" priority="8">
+    <cfRule type="expression" dxfId="58" priority="8">
       <formula>K7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="95" priority="9">
+    <cfRule type="expression" dxfId="57" priority="9">
       <formula>OR(K7="Não atende",K7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O7:O34">
-    <cfRule type="expression" dxfId="94" priority="10">
+    <cfRule type="expression" dxfId="56" priority="10">
       <formula>O7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="93" priority="11">
+    <cfRule type="expression" dxfId="55" priority="11">
       <formula>O7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="92" priority="12">
+    <cfRule type="expression" dxfId="54" priority="12">
       <formula>OR(O7="Não atende",O7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S7:S34">
-    <cfRule type="expression" dxfId="91" priority="13">
+    <cfRule type="expression" dxfId="53" priority="13">
       <formula>S7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="90" priority="14">
+    <cfRule type="expression" dxfId="52" priority="14">
       <formula>S7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="89" priority="15">
+    <cfRule type="expression" dxfId="51" priority="15">
       <formula>OR(S7="Não atende",S7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W7:W34">
-    <cfRule type="expression" dxfId="88" priority="16">
+    <cfRule type="expression" dxfId="50" priority="16">
       <formula>W7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="87" priority="17">
+    <cfRule type="expression" dxfId="49" priority="17">
       <formula>W7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="86" priority="18">
+    <cfRule type="expression" dxfId="48" priority="18">
       <formula>OR(W7="Não atende",W7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -12322,7 +12050,7 @@
         <v>150</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>313</v>
@@ -12332,10 +12060,10 @@
       </c>
       <c r="F31" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="G31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="H31" s="5" t="s">
         <v>317</v>
@@ -12345,11 +12073,11 @@
       </c>
       <c r="J31" s="3">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K31" s="3">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="L31" s="3" t="s">
         <v>96</v>
@@ -12489,24 +12217,24 @@
     <mergeCell ref="K4:L4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C34">
-    <cfRule type="expression" dxfId="85" priority="1">
+    <cfRule type="expression" dxfId="47" priority="1">
       <formula>C7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="84" priority="2">
+    <cfRule type="expression" dxfId="46" priority="2">
       <formula>C7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="83" priority="3">
+    <cfRule type="expression" dxfId="45" priority="3">
       <formula>OR(C7="Não atende",C7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:G34">
-    <cfRule type="expression" dxfId="82" priority="4">
+    <cfRule type="expression" dxfId="44" priority="4">
       <formula>G7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="81" priority="5">
+    <cfRule type="expression" dxfId="43" priority="5">
       <formula>G7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="80" priority="6">
+    <cfRule type="expression" dxfId="42" priority="6">
       <formula>OR(G7="Não atende",G7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15478,7 +15206,7 @@
         <v>0</v>
       </c>
       <c r="S31" s="3" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="T31" s="5" t="s">
         <v>353</v>
@@ -15488,7 +15216,7 @@
       </c>
       <c r="V31" s="3">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W31" s="3" t="s">
         <v>524</v>
@@ -15504,7 +15232,7 @@
         <v>0</v>
       </c>
       <c r="AA31" s="3" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="AB31" s="5" t="s">
         <v>353</v>
@@ -15514,11 +15242,11 @@
       </c>
       <c r="AD31" s="3">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AE31" s="3">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AF31" s="3" t="s">
         <v>96</v>
@@ -15857,79 +15585,79 @@
     <mergeCell ref="AE4:AF4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C34">
-    <cfRule type="expression" dxfId="79" priority="91">
+    <cfRule type="expression" dxfId="41" priority="91">
       <formula>C7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="78" priority="92">
+    <cfRule type="expression" dxfId="40" priority="92">
       <formula>C7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="77" priority="93">
+    <cfRule type="expression" dxfId="39" priority="93">
       <formula>OR(C7="Não atende",C7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:G34">
-    <cfRule type="expression" dxfId="76" priority="64">
+    <cfRule type="expression" dxfId="38" priority="64">
       <formula>G7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="75" priority="65">
+    <cfRule type="expression" dxfId="37" priority="65">
       <formula>G7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="74" priority="66">
+    <cfRule type="expression" dxfId="36" priority="66">
       <formula>OR(G7="Não atende",G7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K7:K34">
-    <cfRule type="expression" dxfId="73" priority="61">
+    <cfRule type="expression" dxfId="35" priority="61">
       <formula>K7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="72" priority="62">
+    <cfRule type="expression" dxfId="34" priority="62">
       <formula>K7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="71" priority="63">
+    <cfRule type="expression" dxfId="33" priority="63">
       <formula>OR(K7="Não atende",K7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O7:O34">
-    <cfRule type="expression" dxfId="70" priority="46">
+    <cfRule type="expression" dxfId="32" priority="46">
       <formula>O7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="69" priority="47">
+    <cfRule type="expression" dxfId="31" priority="47">
       <formula>O7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="68" priority="48">
+    <cfRule type="expression" dxfId="30" priority="48">
       <formula>OR(O7="Não atende",O7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S7:S34">
-    <cfRule type="expression" dxfId="67" priority="25">
+    <cfRule type="expression" dxfId="29" priority="25">
       <formula>S7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="66" priority="26">
+    <cfRule type="expression" dxfId="28" priority="26">
       <formula>S7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="65" priority="27">
+    <cfRule type="expression" dxfId="27" priority="27">
       <formula>OR(S7="Não atende",S7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W7:W34">
-    <cfRule type="expression" dxfId="64" priority="13">
+    <cfRule type="expression" dxfId="26" priority="13">
       <formula>W7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="63" priority="14">
+    <cfRule type="expression" dxfId="25" priority="14">
       <formula>W7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="62" priority="15">
+    <cfRule type="expression" dxfId="24" priority="15">
       <formula>OR(W7="Não atende",W7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA7:AA34">
-    <cfRule type="expression" dxfId="61" priority="1">
+    <cfRule type="expression" dxfId="23" priority="1">
       <formula>AA7="Atende"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="60" priority="2">
+    <cfRule type="expression" dxfId="22" priority="2">
       <formula>AA7="Parcial"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="59" priority="3">
+    <cfRule type="expression" dxfId="21" priority="3">
       <formula>OR(AA7="Não atende",AA7="Sem evidência")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18128,7 +17856,7 @@
         <v>404</v>
       </c>
       <c r="I31" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="J31" s="5" t="s">
         <v>418</v>
@@ -18137,7 +17865,7 @@
         <v>406</v>
       </c>
       <c r="L31" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="M31" s="5" t="s">
         <v>476</v>
@@ -18155,7 +17883,7 @@
         <v>410</v>
       </c>
       <c r="R31" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="S31" s="5" t="s">
         <v>494</v>
@@ -18164,7 +17892,7 @@
         <v>412</v>
       </c>
       <c r="U31" s="3" t="s">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="V31" s="5" t="s">
         <v>442</v>
@@ -18174,7 +17902,7 @@
       </c>
       <c r="X31" s="3">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Y31" s="3" t="s">
         <v>96</v>
@@ -18430,212 +18158,80 @@
     <mergeCell ref="X4:Y4"/>
   </mergeCells>
   <conditionalFormatting sqref="C7:C34">
-    <cfRule type="expression" dxfId="58" priority="37">
+    <cfRule type="expression" dxfId="20" priority="37">
       <formula>C7="Sim"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="38">
+    <cfRule type="expression" dxfId="19" priority="38">
       <formula>C7="Não"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="39">
+    <cfRule type="expression" dxfId="18" priority="39">
       <formula>C7="Sem evidência"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F7:F34">
-    <cfRule type="expression" dxfId="55" priority="40">
+    <cfRule type="expression" dxfId="17" priority="40">
       <formula>F7="Sim"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="54" priority="41">
+    <cfRule type="expression" dxfId="16" priority="41">
       <formula>F7="Não"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="53" priority="42">
+    <cfRule type="expression" dxfId="15" priority="42">
       <formula>F7="Sem evidência"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I7:I34">
-    <cfRule type="expression" dxfId="52" priority="43">
+    <cfRule type="expression" dxfId="14" priority="43">
       <formula>I7="Sim"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="51" priority="44">
+    <cfRule type="expression" dxfId="13" priority="44">
       <formula>I7="Não"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="50" priority="45">
+    <cfRule type="expression" dxfId="12" priority="45">
       <formula>I7="Sem evidência"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L7:L34">
-    <cfRule type="expression" dxfId="49" priority="46">
+    <cfRule type="expression" dxfId="11" priority="46">
       <formula>L7="Sim"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="48" priority="47">
+    <cfRule type="expression" dxfId="10" priority="47">
       <formula>L7="Não"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="47" priority="48">
+    <cfRule type="expression" dxfId="9" priority="48">
       <formula>L7="Sem evidência"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O30 O32 O7:O28">
-    <cfRule type="expression" dxfId="46" priority="49">
+  <conditionalFormatting sqref="O7:O34">
+    <cfRule type="expression" dxfId="8" priority="27">
+      <formula>O7="Sem evidência"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="7" priority="25">
       <formula>O7="Sim"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="45" priority="50">
+    <cfRule type="expression" dxfId="6" priority="26">
       <formula>O7="Não"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="44" priority="51">
-      <formula>O7="Sem evidência"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R7:R34">
+    <cfRule type="expression" dxfId="5" priority="15">
+      <formula>R7="Sem evidência"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="13">
+      <formula>R7="Sim"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="3" priority="14">
+      <formula>R7="Não"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R30 R32 R7:R28">
-    <cfRule type="expression" dxfId="43" priority="52">
-      <formula>R7="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="42" priority="53">
-      <formula>R7="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="41" priority="54">
-      <formula>R7="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U30 U32 U7:U28">
-    <cfRule type="expression" dxfId="40" priority="55">
-      <formula>U7="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="39" priority="56">
+  <conditionalFormatting sqref="U7:U34">
+    <cfRule type="expression" dxfId="2" priority="2">
       <formula>U7="Não"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="57">
+    <cfRule type="expression" dxfId="1" priority="3">
       <formula>U7="Sem evidência"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O29">
-    <cfRule type="expression" dxfId="35" priority="34">
-      <formula>O29="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="34" priority="35">
-      <formula>O29="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="33" priority="36">
-      <formula>O29="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O31">
-    <cfRule type="expression" dxfId="32" priority="31">
-      <formula>O31="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="31" priority="32">
-      <formula>O31="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="30" priority="33">
-      <formula>O31="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O33">
-    <cfRule type="expression" dxfId="29" priority="28">
-      <formula>O33="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="29">
-      <formula>O33="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="27" priority="30">
-      <formula>O33="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O34">
-    <cfRule type="expression" dxfId="26" priority="25">
-      <formula>O34="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="25" priority="26">
-      <formula>O34="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="27">
-      <formula>O34="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R29">
-    <cfRule type="expression" dxfId="23" priority="22">
-      <formula>R29="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="23">
-      <formula>R29="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="21" priority="24">
-      <formula>R29="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R31">
-    <cfRule type="expression" dxfId="20" priority="19">
-      <formula>R31="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="19" priority="20">
-      <formula>R31="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="21">
-      <formula>R31="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R33">
-    <cfRule type="expression" dxfId="17" priority="16">
-      <formula>R33="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="17">
-      <formula>R33="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="15" priority="18">
-      <formula>R33="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R34">
-    <cfRule type="expression" dxfId="14" priority="13">
-      <formula>R34="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="13" priority="14">
-      <formula>R34="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="15">
-      <formula>R34="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U29">
-    <cfRule type="expression" dxfId="11" priority="10">
-      <formula>U29="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="11">
-      <formula>U29="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="9" priority="12">
-      <formula>U29="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U31">
-    <cfRule type="expression" dxfId="8" priority="7">
-      <formula>U31="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="7" priority="8">
-      <formula>U31="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="9">
-      <formula>U31="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U33">
-    <cfRule type="expression" dxfId="5" priority="4">
-      <formula>U33="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="5">
-      <formula>U33="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="3" priority="6">
-      <formula>U33="Sem evidência"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U34">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>U34="Sim"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>U34="Não"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="3">
-      <formula>U34="Sem evidência"</formula>
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>U7="Sim"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -18904,7 +18500,7 @@
       </c>
       <c r="S6">
         <f>COUNTIF(M5:M32,"Instituída")</f>
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.3">
@@ -18975,10 +18571,10 @@
       </c>
       <c r="S7">
         <f>COUNTIF(M5:M32,"Não instituída")</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>105</v>
       </c>
@@ -19188,7 +18784,7 @@
       </c>
       <c r="S10">
         <f>COUNTIF(O5:O32,"*satisfatória*")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.3">
@@ -20293,7 +19889,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>147</v>
       </c>
@@ -20366,62 +19962,62 @@
       </c>
       <c r="C29" s="3">
         <f>'01_Institucionalização'!G31</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="D29" s="3">
         <f>'02_Autonomia'!W31</f>
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E29" s="3">
         <f>'03_Imparcialidade'!K31</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F29" s="3">
         <f>'04_Acessibilidade'!AA31</f>
-        <v>0</v>
+        <v>13.5</v>
       </c>
       <c r="G29" s="3">
         <f>'05_Transparência'!K31</f>
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="H29" s="3">
         <f>'06_Integração Tec'!AE31</f>
-        <v>0</v>
-      </c>
-      <c r="I29" s="3" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="3" t="str">
+        <v>4</v>
+      </c>
+      <c r="I29" s="3">
+        <f t="shared" si="0"/>
+        <v>77.5</v>
+      </c>
+      <c r="J29" s="3">
         <f>IF(M29&lt;&gt;"Instituída","",'07_Maturidade'!X31)</f>
-        <v/>
-      </c>
-      <c r="K29" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="K29" s="3">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="L29" s="3" t="str">
+        <v>5</v>
+      </c>
+      <c r="L29" s="3">
         <f t="shared" si="2"/>
-        <v/>
+        <v>82.5</v>
       </c>
       <c r="M29" s="3" t="str">
         <f>'01_Institucionalização'!H31</f>
-        <v>Não instituída</v>
+        <v>Instituída</v>
       </c>
       <c r="N29" s="3" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>Não</v>
       </c>
       <c r="O29" s="3" t="str">
         <f t="shared" si="4"/>
-        <v>Não instituída</v>
+        <v>Instituída — aderência satisfatória</v>
       </c>
       <c r="P29" s="3" t="str">
         <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.3">
+        <v>Bônus integralmente aplicado</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>151</v>
       </c>

</xml_diff>

<commit_message>
feat: navegação por sub-abas de perguntas, contenção da tabela e tooltips acessíveis
</commit_message>
<xml_diff>
--- a/DADOS.xlsx
+++ b/DADOS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://justicagovbr-my.sharepoint.com/personal/marcelo_cortez_mj_gov_br1/Documents/1. SENAPPEN/2. OUVIDORIA/GITHUB/PARAMETROS MINIMOS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="523" documentId="11_C2318B871671820C540791CC0C0EFCB85A7F69AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDBF98C4-2906-4A1F-8597-21E0CDC6E6F6}"/>
+  <xr:revisionPtr revIDLastSave="525" documentId="11_C2318B871671820C540791CC0C0EFCB85A7F69AA" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67BFA272-BA4A-4042-BCB2-163FBB162495}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="00_Metodologia" sheetId="1" r:id="rId1"/>

</xml_diff>